<commit_message>
feat(examples): the sample workbook carries an entity graph
The xlsx sample gains entity, parent entity, primary keyword, anchors
and page type over eight menu rows, so AutoDetect opens it fully mapped
and an import of it leaves a graph of eight entities and seven parent
edges behind. The csv keeps its three columns as the minimal case.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sitemap-import-example.xlsx
+++ b/examples/sitemap-import-example.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>path</t>
   </si>
@@ -22,210 +22,174 @@
     <t>title</t>
   </si>
   <si>
+    <t>primary keyword</t>
+  </si>
+  <si>
     <t>keywords</t>
   </si>
   <si>
-    <t>/menu</t>
+    <t>entity</t>
+  </si>
+  <si>
+    <t>parent entity</t>
+  </si>
+  <si>
+    <t>anchors</t>
+  </si>
+  <si>
+    <t>page type</t>
+  </si>
+  <si>
+    <t>/menu/</t>
   </si>
   <si>
     <t>Our Menu</t>
   </si>
   <si>
+    <t>restaurant menu</t>
+  </si>
+  <si>
     <t>menu,food,dishes</t>
   </si>
   <si>
-    <t>/menu/appetizers</t>
+    <t>Menu</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>our menu,the menu</t>
+  </si>
+  <si>
+    <t>hub</t>
+  </si>
+  <si>
+    <t>/menu/appetizers/</t>
   </si>
   <si>
     <t>Appetizers</t>
   </si>
   <si>
+    <t>appetizers</t>
+  </si>
+  <si>
     <t>appetizers,starters</t>
   </si>
   <si>
-    <t>/menu/appetizers/soups</t>
-  </si>
-  <si>
-    <t>Soups</t>
-  </si>
-  <si>
-    <t>soups,hot,comfort</t>
-  </si>
-  <si>
-    <t>/menu/appetizers/salads</t>
-  </si>
-  <si>
-    <t>Salads</t>
-  </si>
-  <si>
-    <t>salads,fresh,healthy</t>
-  </si>
-  <si>
-    <t>/menu/main-courses</t>
+    <t>category</t>
+  </si>
+  <si>
+    <t>/menu/main-courses/</t>
   </si>
   <si>
     <t>Main Courses</t>
   </si>
   <si>
+    <t>main courses</t>
+  </si>
+  <si>
     <t>main,entrees,dinner</t>
   </si>
   <si>
-    <t>/menu/main-courses/steaks</t>
+    <t>main courses,entrees</t>
+  </si>
+  <si>
+    <t>/menu/main-courses/steaks/</t>
   </si>
   <si>
     <t>Steaks</t>
   </si>
   <si>
+    <t>grilled steaks</t>
+  </si>
+  <si>
     <t>steaks,beef,grilled</t>
   </si>
   <si>
-    <t>/menu/main-courses/seafood</t>
+    <t>steaks,grilled steaks</t>
+  </si>
+  <si>
+    <t>guide</t>
+  </si>
+  <si>
+    <t>/menu/main-courses/seafood/</t>
   </si>
   <si>
     <t>Seafood</t>
   </si>
   <si>
+    <t>fresh seafood</t>
+  </si>
+  <si>
     <t>seafood,fish,shrimp</t>
   </si>
   <si>
-    <t>/menu/main-courses/pasta</t>
+    <t>seafood,fresh seafood</t>
+  </si>
+  <si>
+    <t>/menu/main-courses/pasta/</t>
   </si>
   <si>
     <t>Pasta</t>
   </si>
   <si>
+    <t>handmade pasta</t>
+  </si>
+  <si>
     <t>pasta,italian,noodles</t>
   </si>
   <si>
-    <t>/menu/desserts</t>
+    <t>pasta,handmade pasta</t>
+  </si>
+  <si>
+    <t>/menu/desserts/</t>
   </si>
   <si>
     <t>Desserts</t>
   </si>
   <si>
+    <t>house desserts</t>
+  </si>
+  <si>
     <t>desserts,sweets,cake</t>
   </si>
   <si>
-    <t>/menu/drinks</t>
+    <t>desserts,sweets</t>
+  </si>
+  <si>
+    <t>/menu/drinks/</t>
   </si>
   <si>
     <t>Drinks</t>
   </si>
   <si>
+    <t>drinks and cocktails</t>
+  </si>
+  <si>
     <t>drinks,beverages,cocktails</t>
   </si>
   <si>
-    <t>/reservations</t>
-  </si>
-  <si>
-    <t>Reservations</t>
-  </si>
-  <si>
-    <t>reservations,booking,table</t>
-  </si>
-  <si>
-    <t>/reservations/private-events</t>
-  </si>
-  <si>
-    <t>Private Events</t>
-  </si>
-  <si>
-    <t>events,parties,catering</t>
-  </si>
-  <si>
-    <t>/locations</t>
-  </si>
-  <si>
-    <t>Our Locations</t>
-  </si>
-  <si>
-    <t>locations,restaurants,addresses</t>
-  </si>
-  <si>
-    <t>/locations/downtown</t>
-  </si>
-  <si>
-    <t>Downtown</t>
-  </si>
-  <si>
-    <t>downtown,city,central</t>
-  </si>
-  <si>
-    <t>/locations/suburbs</t>
-  </si>
-  <si>
-    <t>Suburbs</t>
-  </si>
-  <si>
-    <t>suburbs,family,parking</t>
-  </si>
-  <si>
-    <t>/gift-cards</t>
-  </si>
-  <si>
-    <t>Gift Cards</t>
-  </si>
-  <si>
-    <t>gifts,cards,presents</t>
-  </si>
-  <si>
-    <t>/careers</t>
-  </si>
-  <si>
-    <t>Join Our Team</t>
-  </si>
-  <si>
-    <t>careers,jobs,employment</t>
-  </si>
-  <si>
-    <t>/careers/kitchen</t>
-  </si>
-  <si>
-    <t>Kitchen Positions</t>
-  </si>
-  <si>
-    <t>chef,cook,kitchen</t>
-  </si>
-  <si>
-    <t>/careers/front-of-house</t>
-  </si>
-  <si>
-    <t>Front of House</t>
-  </si>
-  <si>
-    <t>server,host,bartender</t>
+    <t>drinks,cocktails</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE0E0E0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -240,11 +204,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="false">
-      <alignment/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,230 +475,239 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col customWidth="true" max="1" min="1" width="30"/>
-    <col customWidth="true" max="2" min="2" width="20"/>
-    <col customWidth="true" max="3" min="3" width="30"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
         <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>54</v>
-      </c>
-      <c r="B19" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test(e2e): the whole loop against the docker WordPress stack
internal/e2e composes the real application over a scripted model,
syncs the docker site, imports the sample workbook, generates five
guide pages as drafts and waits on ListEvents. It then reads the live
site through the companion plugin: five drafts under /menu/, each
linking to its parent with its SEO meta written, the two parent pages
relinked to their new children, realized edges in the site overview,
compliance 1.0 in every final report and a backup that round trips.
`task e2e:full` brings the stack up and runs it.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sitemap-import-example.xlsx
+++ b/examples/sitemap-import-example.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>path</t>
   </si>
@@ -58,7 +58,7 @@
     <t/>
   </si>
   <si>
-    <t>our menu,the menu</t>
+    <t>our menu|the menu</t>
   </si>
   <si>
     <t>hub</t>
@@ -76,6 +76,9 @@
     <t>appetizers,starters</t>
   </si>
   <si>
+    <t>appetizers|starters</t>
+  </si>
+  <si>
     <t>category</t>
   </si>
   <si>
@@ -91,7 +94,7 @@
     <t>main,entrees,dinner</t>
   </si>
   <si>
-    <t>main courses,entrees</t>
+    <t>main courses|entrees</t>
   </si>
   <si>
     <t>/menu/main-courses/steaks/</t>
@@ -106,7 +109,7 @@
     <t>steaks,beef,grilled</t>
   </si>
   <si>
-    <t>steaks,grilled steaks</t>
+    <t>steaks|grilled steaks</t>
   </si>
   <si>
     <t>guide</t>
@@ -124,7 +127,7 @@
     <t>seafood,fish,shrimp</t>
   </si>
   <si>
-    <t>seafood,fresh seafood</t>
+    <t>seafood|fresh seafood</t>
   </si>
   <si>
     <t>/menu/main-courses/pasta/</t>
@@ -139,7 +142,7 @@
     <t>pasta,italian,noodles</t>
   </si>
   <si>
-    <t>pasta,handmade pasta</t>
+    <t>pasta|handmade pasta</t>
   </si>
   <si>
     <t>/menu/desserts/</t>
@@ -154,7 +157,7 @@
     <t>desserts,sweets,cake</t>
   </si>
   <si>
-    <t>desserts,sweets</t>
+    <t>desserts|sweets</t>
   </si>
   <si>
     <t>/menu/drinks/</t>
@@ -169,7 +172,7 @@
     <t>drinks,beverages,cocktails</t>
   </si>
   <si>
-    <t>drinks,cocktails</t>
+    <t>drinks|cocktails</t>
   </si>
 </sst>
 </file>
@@ -548,166 +551,166 @@
         <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
         <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
       </c>
       <c r="F4" t="s">
         <v>12</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" t="s">
         <v>28</v>
       </c>
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" t="s">
-        <v>27</v>
-      </c>
       <c r="F5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" t="s">
         <v>32</v>
-      </c>
-      <c r="B6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" t="s">
         <v>39</v>
       </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s">
-        <v>38</v>
-      </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
         <v>44</v>
-      </c>
-      <c r="D8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" t="s">
-        <v>43</v>
       </c>
       <c r="F8" t="s">
         <v>12</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" t="s">
         <v>49</v>
-      </c>
-      <c r="D9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" t="s">
-        <v>48</v>
       </c>
       <c r="F9" t="s">
         <v>12</v>
       </c>
       <c r="G9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>